<commit_message>
Up to Author's Note
</commit_message>
<xml_diff>
--- a/scripts/atrioc-vods.xlsx
+++ b/scripts/atrioc-vods.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de23bfdcd6216b10/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8854" documentId="8_{AB2BEB25-6301-4E07-BA40-B9523C5F4B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6F58257-1A88-47D4-8CDF-301A38738724}"/>
+  <xr:revisionPtr revIDLastSave="8858" documentId="8_{AB2BEB25-6301-4E07-BA40-B9523C5F4B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{716F2E84-7925-48E9-BD89-091FA652F761}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7BDED62C-F0DC-47C1-9BFD-0430D6E1AEAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{7BDED62C-F0DC-47C1-9BFD-0430D6E1AEAA}"/>
   </bookViews>
   <sheets>
     <sheet name="vods" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4605" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4607" uniqueCount="937">
   <si>
     <t>video_id</t>
   </si>
@@ -2982,6 +2982,9 @@
   </si>
   <si>
     <t>Did I Meet My 2025 Goals?</t>
+  </si>
+  <si>
+    <t>osrs</t>
   </si>
 </sst>
 </file>
@@ -3165,8 +3168,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F8CC73E4-F3CC-4C29-B708-968A8C2A6FA4}" name="Table5810" displayName="Table5810" ref="A1:C110" totalsRowShown="0">
-  <autoFilter ref="A1:C110" xr:uid="{F8CC73E4-F3CC-4C29-B708-968A8C2A6FA4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F8CC73E4-F3CC-4C29-B708-968A8C2A6FA4}" name="Table5810" displayName="Table5810" ref="A1:C111" totalsRowShown="0">
+  <autoFilter ref="A1:C111" xr:uid="{F8CC73E4-F3CC-4C29-B708-968A8C2A6FA4}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6DCE3215-DFFE-4FCE-92A2-DFC31EC00185}" name="video_id"/>
     <tableColumn id="2" xr3:uid="{23D3B8E5-2F44-4DC8-834D-C9D449D72555}" name="game"/>
@@ -28472,7 +28475,15 @@
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C111" s="2"/>
+      <c r="A111" t="s">
+        <v>923</v>
+      </c>
+      <c r="B111" t="s">
+        <v>936</v>
+      </c>
+      <c r="C111" s="2">
+        <v>63</v>
+      </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C112" s="2"/>
@@ -28509,7 +28520,7 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:A110" xr:uid="{9B2D3CCE-D5A4-498D-8D83-EF30CFA7E8FC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:A111" xr:uid="{9B2D3CCE-D5A4-498D-8D83-EF30CFA7E8FC}">
       <formula1>video_id</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C4 C6:C34 C36:C73" xr:uid="{F23220A0-D767-46E3-A31E-906F41C8AE85}">

</xml_diff>